<commit_message>
Regenerate latest output after structural autosizing
Synchronize outputs/latest with the structurally closed autosized configuration.
</commit_message>
<xml_diff>
--- a/outputs/latest/details/params.xlsx
+++ b/outputs/latest/details/params.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Parameters" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D213"/>
+  <dimension ref="A1:D236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -811,7 +811,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>135</v>
+        <v>149</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>3374.2</v>
+        <v>3600</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -913,7 +913,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1687.1</v>
+        <v>1800</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -933,7 +933,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>325.8</v>
+        <v>310</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -953,7 +953,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>195.48</v>
+        <v>190</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>266.0699999999999</v>
+        <v>254.8</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -993,7 +993,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>320.3265000000001</v>
+        <v>392.014</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1013,7 +1013,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>386.844</v>
+        <v>455.714</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1033,7 +1033,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>96.86430732488546</v>
+        <v>86.00930732488546</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1053,7 +1053,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>28</v>
+        <v>46.5</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1073,7 +1073,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>0.6</v>
+        <v>0.6129032258064516</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1174,7 +1174,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>NACA4412</t>
+          <t>NACA6415</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1195,7 +1195,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>22.75000000000001</v>
+        <v>32</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1215,7 +1215,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>17.06250000000001</v>
+        <v>30</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1291,11 +1291,11 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>fuselage_longeron_OD</t>
+          <t>wing_primary_spar_layout_OD</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>6.5</v>
+        <v>32</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1311,11 +1311,11 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>fuselage_longeron_boss_OD</t>
+          <t>fuselage_longeron_OD</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>12.5</v>
+        <v>8</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1331,11 +1331,11 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>fuselage_longeron_top_z</t>
+          <t>fuselage_longeron_boss_OD</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>110.7593073248855</v>
+        <v>14</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1351,11 +1351,11 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>fuselage_longeron_bottom_z</t>
+          <t>fuselage_longeron_top_z</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>-110.7593073248855</v>
+        <v>110.0093073248855</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1371,11 +1371,11 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>fuselage_top_z</t>
+          <t>fuselage_longeron_bottom_z</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>114.0093073248855</v>
+        <v>-110.0093073248855</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1391,11 +1391,11 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>wing_drop_from_flush</t>
+          <t>fuselage_top_z</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>3.145000000000009</v>
+        <v>114.0093073248855</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1411,11 +1411,11 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>horizontal_tail_span</t>
+          <t>wing_drop_from_flush</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>868.8000000000001</v>
+        <v>4.750000000000004</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -1431,11 +1431,11 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>horizontal_tail_half_span</t>
+          <t>horizontal_tail_span</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>434.4</v>
+        <v>915.9221570593505</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -1451,11 +1451,11 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>horizontal_tail_root_chord</t>
+          <t>horizontal_tail_half_span</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>218</v>
+        <v>457.9610785296753</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -1471,11 +1471,11 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>horizontal_tail_tip_chord</t>
+          <t>horizontal_tail_root_chord</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>152.6</v>
+        <v>218</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -1491,11 +1491,11 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>horizontal_tail_mac</t>
+          <t>horizontal_tail_tip_chord</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>187.2235294117647</v>
+        <v>152.6</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -1511,11 +1511,11 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>horizontal_tail_le_x</t>
+          <t>horizontal_tail_mac</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>1002.136117647059</v>
+        <v>187.2235294117647</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -1531,11 +1531,11 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>horizontal_tail_ac_x</t>
+          <t>horizontal_tail_le_x</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>1048.942</v>
+        <v>1003.420117647059</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -1551,11 +1551,11 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>horizontal_tail_z</t>
+          <t>horizontal_tail_ac_x</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>96.86430732488546</v>
+        <v>1050.226</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -1571,11 +1571,11 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>horizontal_tail_thickness</t>
+          <t>horizontal_tail_z</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>22</v>
+        <v>86.00930732488546</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -1591,15 +1591,15 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>horizontal_tail_taper_ratio</t>
+          <t>horizontal_tail_thickness</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>0.7</v>
+        <v>26.16</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>unitless</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -1611,17 +1611,15 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>horizontal_tail_NACA</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>NACA0012</t>
-        </is>
+          <t>horizontal_tail_taper_ratio</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>0.7</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>unitless</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1633,15 +1631,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>horizontal_tail_primary_spar_OD</t>
-        </is>
-      </c>
-      <c r="B61" t="n">
-        <v>9.500000000000005</v>
+          <t>horizontal_tail_NACA</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>NACA0012</t>
+        </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>String</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -1653,11 +1653,11 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>horizontal_tail_primary_spar_ID</t>
+          <t>horizontal_tail_primary_spar_OD</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>7.125000000000004</v>
+        <v>10</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -1673,11 +1673,11 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>horizontal_tail_secondary_spar_OD</t>
+          <t>horizontal_tail_primary_spar_ID</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -1693,15 +1693,15 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>vertical_tail_count</t>
+          <t>horizontal_tail_secondary_spar_OD</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>unitless</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -1713,15 +1713,15 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>vertical_tail_height</t>
+          <t>vertical_tail_count</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>300</v>
+        <v>2</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>unitless</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -1733,11 +1733,11 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>vertical_tail_root_chord</t>
+          <t>vertical_tail_height</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>148</v>
+        <v>533.0190749553177</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -1753,11 +1753,11 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>vertical_tail_tip_chord</t>
+          <t>vertical_tail_root_chord</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>88.79999999999998</v>
+        <v>148</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -1773,11 +1773,11 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>vertical_tail_le_x</t>
+          <t>vertical_tail_tip_chord</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>991.3753333333334</v>
+        <v>88.79999999999998</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -1793,11 +1793,11 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>vertical_tail_ac_x</t>
+          <t>vertical_tail_le_x</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>1021.592</v>
+        <v>1080.074333333333</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -1813,11 +1813,11 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>vertical_tail_thickness</t>
+          <t>vertical_tail_ac_x</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>12</v>
+        <v>1110.291</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -1833,15 +1833,15 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>vertical_tail_taper_ratio</t>
+          <t>vertical_tail_thickness</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>0.6</v>
+        <v>17.76</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>unitless</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -1853,17 +1853,15 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>vertical_tail_NACA</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>NACA0012</t>
-        </is>
+          <t>vertical_tail_taper_ratio</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>0.6</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>unitless</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -1875,15 +1873,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>vertical_tail_primary_spar_OD</t>
-        </is>
-      </c>
-      <c r="B73" t="n">
-        <v>7.250000000000003</v>
+          <t>vertical_tail_NACA</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>NACA0012</t>
+        </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>String</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -1895,11 +1895,11 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>vertical_tail_primary_spar_ID</t>
+          <t>vertical_tail_primary_spar_OD</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>5.437500000000003</v>
+        <v>10</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
@@ -1915,11 +1915,11 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>vertical_tail_secondary_spar_OD</t>
+          <t>vertical_tail_primary_spar_ID</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
@@ -1935,11 +1935,11 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>boom_length</t>
+          <t>vertical_tail_secondary_spar_OD</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>1003.516</v>
+        <v>4</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
@@ -1955,11 +1955,11 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>boom_start_x</t>
+          <t>boom_length</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>96.48400000000001</v>
+        <v>913.6600000000001</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
@@ -1975,11 +1975,11 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>boom_end_x</t>
+          <t>boom_start_x</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>1100</v>
+        <v>186.34</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
@@ -1995,11 +1995,11 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>boom_left_y</t>
+          <t>boom_end_x</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>-366.9</v>
+        <v>1100</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
@@ -2015,11 +2015,11 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>boom_right_y</t>
+          <t>boom_left_y</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>366.9</v>
+        <v>-373.9</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -2035,11 +2035,11 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>boom_spacing</t>
+          <t>boom_right_y</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>733.8</v>
+        <v>373.9</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
@@ -2055,11 +2055,11 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>boom_z</t>
+          <t>boom_spacing</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>96.86430732488546</v>
+        <v>747.8000000000001</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
@@ -2075,11 +2075,11 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>boom_OD</t>
+          <t>boom_z</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>21.25000000000001</v>
+        <v>86.00930732488546</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -2095,11 +2095,11 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>boom_ID</t>
+          <t>boom_OD</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>17.25000000000001</v>
+        <v>26</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -2115,11 +2115,11 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>lift_motor_front_x</t>
+          <t>boom_ID</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>96.48400000000001</v>
+        <v>24</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -2135,15 +2135,15 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>lift_motor_rear_x</t>
+          <t>landing_legs_enabled</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>675.284</v>
+        <v>1</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>unitless</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2155,11 +2155,11 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>lift_motor_y_abs</t>
+          <t>landing_ground_z</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>366.9</v>
+        <v>-243.1156926751145</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -2175,11 +2175,11 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>lift_motor_z</t>
+          <t>landing_leg_tube_OD</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>127.8893073248855</v>
+        <v>8</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
@@ -2195,11 +2195,11 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>lift_prop_diameter</t>
+          <t>landing_leg_tube_ID</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>558.8</v>
+        <v>6</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
@@ -2215,11 +2215,11 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>lift_prop_pitch</t>
+          <t>landing_leg_sleeve_OD</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>167.64</v>
+        <v>12</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
@@ -2235,17 +2235,15 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>lift_motor_name</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>Tmotor_U8Lite_150kV_P22x6p6_12S</t>
-        </is>
+          <t>landing_leg_sleeve_wall</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>2</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -2257,11 +2255,11 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>lift_motor_OD</t>
+          <t>landing_leg_sizing_length</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>87.09999999999999</v>
+        <v>305.875</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
@@ -2277,11 +2275,11 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>lift_motor_body_length</t>
+          <t>landing_leg_nose_x</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>27.05</v>
+        <v>70</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
@@ -2297,11 +2295,11 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>pusher_motor_x</t>
+          <t>landing_leg_nose_y</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>896.3500000000003</v>
+        <v>0</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
@@ -2317,11 +2315,11 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>pusher_motor_y</t>
+          <t>landing_leg_nose_mount_z</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>0</v>
+        <v>-114.0093073248855</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
@@ -2337,11 +2335,11 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>pusher_motor_z</t>
+          <t>landing_leg_nose_foot_z</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>0</v>
+        <v>-243.1156926751145</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
@@ -2357,11 +2355,11 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>pusher_prop_diameter</t>
+          <t>landing_leg_nose_length</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>381</v>
+        <v>129.1063853502291</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
@@ -2377,11 +2375,11 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>pusher_prop_pitch</t>
+          <t>landing_leg_wing_left_x</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>127</v>
+        <v>455.7139999999999</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
@@ -2397,17 +2395,15 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>pusher_motor_name</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>Tmotor_MN501S_240kV_P15x5_12S</t>
-        </is>
+          <t>landing_leg_wing_left_y</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>-373.9</v>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -2419,11 +2415,11 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>pusher_motor_OD</t>
+          <t>landing_leg_wing_left_mount_z</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>55.59999999999999</v>
+        <v>62.75930732488547</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
@@ -2439,11 +2435,11 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>pusher_motor_body_length</t>
+          <t>landing_leg_wing_left_foot_z</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>33.9</v>
+        <v>-243.1156926751145</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
@@ -2459,11 +2455,11 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>payload_x</t>
+          <t>landing_leg_wing_left_length</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>103.5</v>
+        <v>305.875</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
@@ -2479,11 +2475,11 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>payload_y</t>
+          <t>landing_leg_wing_right_x</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>0</v>
+        <v>455.7139999999999</v>
       </c>
       <c r="C103" t="inlineStr">
         <is>
@@ -2499,11 +2495,11 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>payload_z</t>
+          <t>landing_leg_wing_right_y</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>-28.00930732488547</v>
+        <v>373.9</v>
       </c>
       <c r="C104" t="inlineStr">
         <is>
@@ -2519,11 +2515,11 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>payload_length</t>
+          <t>landing_leg_wing_right_mount_z</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>53</v>
+        <v>62.75930732488547</v>
       </c>
       <c r="C105" t="inlineStr">
         <is>
@@ -2539,11 +2535,11 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>payload_width</t>
+          <t>landing_leg_wing_right_foot_z</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>80</v>
+        <v>-243.1156926751145</v>
       </c>
       <c r="C106" t="inlineStr">
         <is>
@@ -2559,11 +2555,11 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>payload_height</t>
+          <t>landing_leg_wing_right_length</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>80</v>
+        <v>305.875</v>
       </c>
       <c r="C107" t="inlineStr">
         <is>
@@ -2579,11 +2575,11 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>battery_x</t>
+          <t>lift_motor_front_x</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>221.5</v>
+        <v>186.34</v>
       </c>
       <c r="C108" t="inlineStr">
         <is>
@@ -2599,11 +2595,11 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>battery_y</t>
+          <t>lift_motor_rear_x</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>0</v>
+        <v>765.14</v>
       </c>
       <c r="C109" t="inlineStr">
         <is>
@@ -2619,11 +2615,11 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>battery_z</t>
+          <t>lift_motor_y_abs</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>60.29069267511453</v>
+        <v>373.9</v>
       </c>
       <c r="C110" t="inlineStr">
         <is>
@@ -2639,11 +2635,11 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>battery_length</t>
+          <t>lift_motor_z</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>163</v>
+        <v>56.28430732488547</v>
       </c>
       <c r="C111" t="inlineStr">
         <is>
@@ -2659,11 +2655,11 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>battery_width</t>
+          <t>lift_prop_diameter</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>92</v>
+        <v>558.8</v>
       </c>
       <c r="C112" t="inlineStr">
         <is>
@@ -2679,11 +2675,11 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>battery_height</t>
+          <t>lift_prop_pitch</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>51</v>
+        <v>167.64</v>
       </c>
       <c r="C113" t="inlineStr">
         <is>
@@ -2699,15 +2695,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>fuel_cell_x</t>
-        </is>
-      </c>
-      <c r="B114" t="n">
-        <v>255.25</v>
+          <t>lift_motor_name</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Tmotor_U8Lite_150kV_P22x6p6_12S</t>
+        </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>String</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -2719,11 +2717,11 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>fuel_cell_y</t>
+          <t>lift_motor_OD</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>0</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="C115" t="inlineStr">
         <is>
@@ -2739,11 +2737,11 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>fuel_cell_z</t>
+          <t>lift_motor_body_length</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>-28.10930732488547</v>
+        <v>27.05</v>
       </c>
       <c r="C116" t="inlineStr">
         <is>
@@ -2759,11 +2757,11 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>fuel_cell_length</t>
+          <t>pusher_motor_x</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>230.5</v>
+        <v>896.3500000000003</v>
       </c>
       <c r="C117" t="inlineStr">
         <is>
@@ -2779,11 +2777,11 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>fuel_cell_width</t>
+          <t>pusher_motor_y</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>108.4</v>
+        <v>0</v>
       </c>
       <c r="C118" t="inlineStr">
         <is>
@@ -2799,11 +2797,11 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>fuel_cell_height</t>
+          <t>pusher_motor_z</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>119.8</v>
+        <v>0</v>
       </c>
       <c r="C119" t="inlineStr">
         <is>
@@ -2819,11 +2817,11 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>fuel_cell_control_box_x</t>
+          <t>pusher_prop_diameter</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>414.1</v>
+        <v>457.2</v>
       </c>
       <c r="C120" t="inlineStr">
         <is>
@@ -2839,11 +2837,11 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>fuel_cell_control_box_y</t>
+          <t>pusher_prop_pitch</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>0</v>
+        <v>254</v>
       </c>
       <c r="C121" t="inlineStr">
         <is>
@@ -2859,15 +2857,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>fuel_cell_control_box_z</t>
-        </is>
-      </c>
-      <c r="B122" t="n">
-        <v>57.36569267511453</v>
+          <t>pusher_motor_name</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Tmotor_MN501S_160kV_P18x10_12S</t>
+        </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>String</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -2879,11 +2879,11 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>fuel_cell_control_box_length</t>
+          <t>pusher_motor_OD</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>202.2</v>
+        <v>55.59999999999999</v>
       </c>
       <c r="C123" t="inlineStr">
         <is>
@@ -2899,11 +2899,11 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>fuel_cell_control_box_width</t>
+          <t>pusher_motor_body_length</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>107</v>
+        <v>33.9</v>
       </c>
       <c r="C124" t="inlineStr">
         <is>
@@ -2919,11 +2919,11 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>fuel_cell_control_box_height</t>
+          <t>payload_x</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>45.15000000000001</v>
+        <v>103.5</v>
       </c>
       <c r="C125" t="inlineStr">
         <is>
@@ -2939,11 +2939,11 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>hydrogen_cylinder_x</t>
+          <t>payload_y</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>593.0000000000001</v>
+        <v>0</v>
       </c>
       <c r="C126" t="inlineStr">
         <is>
@@ -2959,11 +2959,11 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>hydrogen_cylinder_y</t>
+          <t>payload_z</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>0</v>
+        <v>-33.00930732488546</v>
       </c>
       <c r="C127" t="inlineStr">
         <is>
@@ -2979,11 +2979,11 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>hydrogen_cylinder_z</t>
+          <t>payload_length</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>-30.50930732488547</v>
+        <v>53</v>
       </c>
       <c r="C128" t="inlineStr">
         <is>
@@ -2999,11 +2999,11 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>hydrogen_cylinder_length</t>
+          <t>payload_width</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>425</v>
+        <v>80</v>
       </c>
       <c r="C129" t="inlineStr">
         <is>
@@ -3019,11 +3019,11 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>hydrogen_cylinder_diameter</t>
+          <t>payload_height</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>115</v>
+        <v>80</v>
       </c>
       <c r="C130" t="inlineStr">
         <is>
@@ -3039,11 +3039,11 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>cube_orange_x</t>
+          <t>battery_x</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>82.75</v>
+        <v>221.5</v>
       </c>
       <c r="C131" t="inlineStr">
         <is>
@@ -3059,7 +3059,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>cube_orange_y</t>
+          <t>battery_y</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -3079,11 +3079,11 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>cube_orange_z</t>
+          <t>battery_z</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>30.49069267511453</v>
+        <v>62.29069267511454</v>
       </c>
       <c r="C133" t="inlineStr">
         <is>
@@ -3099,11 +3099,11 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>cube_orange_length</t>
+          <t>battery_length</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>94.5</v>
+        <v>163</v>
       </c>
       <c r="C134" t="inlineStr">
         <is>
@@ -3119,11 +3119,11 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>cube_orange_width</t>
+          <t>battery_width</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>44.3</v>
+        <v>92</v>
       </c>
       <c r="C135" t="inlineStr">
         <is>
@@ -3139,11 +3139,11 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>cube_orange_height</t>
+          <t>battery_height</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="C136" t="inlineStr">
         <is>
@@ -3159,11 +3159,11 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>pdb_x</t>
+          <t>fuel_cell_x</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>565.2</v>
+        <v>255.25</v>
       </c>
       <c r="C137" t="inlineStr">
         <is>
@@ -3179,7 +3179,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>pdb_y</t>
+          <t>fuel_cell_y</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -3199,11 +3199,11 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>pdb_z</t>
+          <t>fuel_cell_z</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>63.54069267511453</v>
+        <v>-33.10930732488546</v>
       </c>
       <c r="C139" t="inlineStr">
         <is>
@@ -3219,11 +3219,11 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>pdb_length</t>
+          <t>fuel_cell_length</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>80</v>
+        <v>230.5</v>
       </c>
       <c r="C140" t="inlineStr">
         <is>
@@ -3239,11 +3239,11 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>pdb_width</t>
+          <t>fuel_cell_width</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>60</v>
+        <v>108.4</v>
       </c>
       <c r="C141" t="inlineStr">
         <is>
@@ -3259,11 +3259,11 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>pdb_height</t>
+          <t>fuel_cell_height</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>23.5</v>
+        <v>119.8</v>
       </c>
       <c r="C142" t="inlineStr">
         <is>
@@ -3279,11 +3279,11 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>pdb2_x</t>
+          <t>fuel_cell_control_box_x</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>655.2000000000002</v>
+        <v>414.1</v>
       </c>
       <c r="C143" t="inlineStr">
         <is>
@@ -3299,7 +3299,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>pdb2_y</t>
+          <t>fuel_cell_control_box_y</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -3319,11 +3319,11 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>pdb2_z</t>
+          <t>fuel_cell_control_box_z</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>63.54069267511453</v>
+        <v>59.36569267511454</v>
       </c>
       <c r="C145" t="inlineStr">
         <is>
@@ -3339,11 +3339,11 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>pdb2_length</t>
+          <t>fuel_cell_control_box_length</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>80</v>
+        <v>202.2</v>
       </c>
       <c r="C146" t="inlineStr">
         <is>
@@ -3359,11 +3359,11 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>pdb2_width</t>
+          <t>fuel_cell_control_box_width</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>60</v>
+        <v>107</v>
       </c>
       <c r="C147" t="inlineStr">
         <is>
@@ -3379,11 +3379,11 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>pdb2_height</t>
+          <t>fuel_cell_control_box_height</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>23.5</v>
+        <v>45.15000000000001</v>
       </c>
       <c r="C148" t="inlineStr">
         <is>
@@ -3399,17 +3399,15 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>fc_cooling_architecture</t>
-        </is>
-      </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>cross_fuselage</t>
-        </is>
+          <t>hydrogen_cylinder_x</t>
+        </is>
+      </c>
+      <c r="B149" t="n">
+        <v>593.0000000000001</v>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -3421,17 +3419,15 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>fc_cooling_fan_flow_direction</t>
-        </is>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>suction_through_stack_to_fan_side</t>
-        </is>
+          <t>hydrogen_cylinder_y</t>
+        </is>
+      </c>
+      <c r="B150" t="n">
+        <v>0</v>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -3443,17 +3439,15 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>fc_cooling_inlet_side</t>
-        </is>
-      </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>left</t>
-        </is>
+          <t>hydrogen_cylinder_z</t>
+        </is>
+      </c>
+      <c r="B151" t="n">
+        <v>-35.50930732488546</v>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -3465,17 +3459,15 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>fc_cooling_exhaust_side</t>
-        </is>
-      </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
+          <t>hydrogen_cylinder_length</t>
+        </is>
+      </c>
+      <c r="B152" t="n">
+        <v>425</v>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -3487,11 +3479,11 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>fc_cooling_inlet_center_x</t>
+          <t>hydrogen_cylinder_diameter</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>255.25</v>
+        <v>115</v>
       </c>
       <c r="C153" t="inlineStr">
         <is>
@@ -3507,11 +3499,11 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>fc_cooling_inlet_center_y</t>
+          <t>cube_orange_x</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>-67.5</v>
+        <v>82.75</v>
       </c>
       <c r="C154" t="inlineStr">
         <is>
@@ -3527,11 +3519,11 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>fc_cooling_inlet_center_z</t>
+          <t>cube_orange_y</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>-28.10930732488547</v>
+        <v>0</v>
       </c>
       <c r="C155" t="inlineStr">
         <is>
@@ -3547,11 +3539,11 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>fc_cooling_inlet_panel_length</t>
+          <t>cube_orange_z</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>170</v>
+        <v>32.49069267511454</v>
       </c>
       <c r="C156" t="inlineStr">
         <is>
@@ -3567,11 +3559,11 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>fc_cooling_inlet_panel_height</t>
+          <t>cube_orange_length</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>105</v>
+        <v>94.5</v>
       </c>
       <c r="C157" t="inlineStr">
         <is>
@@ -3587,15 +3579,15 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>fc_cooling_inlet_slot_count</t>
+          <t>cube_orange_width</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>12</v>
+        <v>44.3</v>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>unitless</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -3607,11 +3599,11 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>fc_cooling_inlet_slot_length</t>
+          <t>cube_orange_height</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>170</v>
+        <v>31</v>
       </c>
       <c r="C159" t="inlineStr">
         <is>
@@ -3627,11 +3619,11 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>fc_cooling_inlet_slot_width</t>
+          <t>pdb_x</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>6</v>
+        <v>565.2</v>
       </c>
       <c r="C160" t="inlineStr">
         <is>
@@ -3647,11 +3639,11 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>fc_cooling_inlet_slot_gap</t>
+          <t>pdb_y</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C161" t="inlineStr">
         <is>
@@ -3667,11 +3659,11 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>fc_cooling_inlet_recess_depth</t>
+          <t>pdb_z</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>8</v>
+        <v>58.54069267511454</v>
       </c>
       <c r="C162" t="inlineStr">
         <is>
@@ -3687,11 +3679,11 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>fc_cooling_inlet_ramp_length</t>
+          <t>pdb_length</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>170</v>
+        <v>80</v>
       </c>
       <c r="C163" t="inlineStr">
         <is>
@@ -3707,15 +3699,15 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>fc_cooling_inlet_ramp_angle</t>
+          <t>pdb_width</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>2.694284289856101</v>
+        <v>60</v>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>deg</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -3727,15 +3719,15 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>fc_cooling_inlet_sidewall_angle</t>
+          <t>pdb_height</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>7</v>
+        <v>23.5</v>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>deg</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -3747,11 +3739,11 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>fc_cooling_inlet_lip_radius</t>
+          <t>pdb2_x</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>2</v>
+        <v>655.2000000000002</v>
       </c>
       <c r="C166" t="inlineStr">
         <is>
@@ -3767,11 +3759,11 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>fc_cooling_exhaust_center_x</t>
+          <t>pdb2_y</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>255.25</v>
+        <v>0</v>
       </c>
       <c r="C167" t="inlineStr">
         <is>
@@ -3787,11 +3779,11 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>fc_cooling_exhaust_center_y</t>
+          <t>pdb2_z</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>67.5</v>
+        <v>58.54069267511454</v>
       </c>
       <c r="C168" t="inlineStr">
         <is>
@@ -3807,11 +3799,11 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>fc_cooling_exhaust_center_z</t>
+          <t>pdb2_length</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>-28.10930732488547</v>
+        <v>80</v>
       </c>
       <c r="C169" t="inlineStr">
         <is>
@@ -3827,11 +3819,11 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>fc_cooling_exhaust_panel_length</t>
+          <t>pdb2_width</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>180</v>
+        <v>60</v>
       </c>
       <c r="C170" t="inlineStr">
         <is>
@@ -3847,11 +3839,11 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>fc_cooling_exhaust_panel_height</t>
+          <t>pdb2_height</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>111</v>
+        <v>23.5</v>
       </c>
       <c r="C171" t="inlineStr">
         <is>
@@ -3867,15 +3859,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>fc_cooling_exhaust_slot_count</t>
-        </is>
-      </c>
-      <c r="B172" t="n">
-        <v>12</v>
+          <t>fc_cooling_architecture</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>cross_fuselage</t>
+        </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>unitless</t>
+          <t>String</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -3887,15 +3881,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>fc_cooling_exhaust_slot_length</t>
-        </is>
-      </c>
-      <c r="B173" t="n">
-        <v>180</v>
+          <t>fc_cooling_fan_flow_direction</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>suction_through_stack_to_fan_side</t>
+        </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>String</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -3907,15 +3903,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>fc_cooling_exhaust_slot_width</t>
-        </is>
-      </c>
-      <c r="B174" t="n">
-        <v>6.5</v>
+          <t>fc_cooling_inlet_side</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>left</t>
+        </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>String</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -3927,15 +3925,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>fc_cooling_exhaust_slot_gap</t>
-        </is>
-      </c>
-      <c r="B175" t="n">
-        <v>3</v>
+          <t>fc_cooling_exhaust_side</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>String</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -3947,11 +3947,11 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>fc_cooling_exhaust_shroud_depth</t>
+          <t>fc_cooling_inlet_center_x</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>10</v>
+        <v>255.25</v>
       </c>
       <c r="C176" t="inlineStr">
         <is>
@@ -3967,15 +3967,15 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>fc_cooling_exhaust_louvre_angle</t>
+          <t>fc_cooling_inlet_center_y</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>15</v>
+        <v>-74.50000000000001</v>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>deg</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -3987,11 +3987,11 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>fc_cooling_exhaust_lip_radius</t>
+          <t>fc_cooling_inlet_center_z</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>2</v>
+        <v>-33.10930732488546</v>
       </c>
       <c r="C178" t="inlineStr">
         <is>
@@ -4007,15 +4007,15 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>fc_cooling_fan_count</t>
+          <t>fc_cooling_inlet_panel_length</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>2</v>
+        <v>170</v>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>unitless</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -4027,11 +4027,11 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>fc_cooling_fan_diameter</t>
+          <t>fc_cooling_inlet_panel_height</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>80</v>
+        <v>105</v>
       </c>
       <c r="C180" t="inlineStr">
         <is>
@@ -4047,15 +4047,15 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>fc_cooling_fan_center_spacing</t>
+          <t>fc_cooling_inlet_slot_count</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>86</v>
+        <v>12</v>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>unitless</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -4067,11 +4067,11 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>fc_cooling_fan_1_center_x</t>
+          <t>fc_cooling_inlet_slot_length</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>212.2500000000001</v>
+        <v>170</v>
       </c>
       <c r="C182" t="inlineStr">
         <is>
@@ -4087,11 +4087,11 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>fc_cooling_fan_2_center_x</t>
+          <t>fc_cooling_inlet_slot_width</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>298.25</v>
+        <v>6</v>
       </c>
       <c r="C183" t="inlineStr">
         <is>
@@ -4107,11 +4107,11 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>fc_cooling_fan_center_y</t>
+          <t>fc_cooling_inlet_slot_gap</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>67.5</v>
+        <v>3</v>
       </c>
       <c r="C184" t="inlineStr">
         <is>
@@ -4127,11 +4127,11 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>fc_cooling_fan_center_z</t>
+          <t>fc_cooling_inlet_recess_depth</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>-28.10930732488547</v>
+        <v>8</v>
       </c>
       <c r="C185" t="inlineStr">
         <is>
@@ -4147,11 +4147,11 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>fc_cooling_inlet_plenum_gap_actual</t>
+          <t>fc_cooling_inlet_ramp_length</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>3.300000000000004</v>
+        <v>170</v>
       </c>
       <c r="C186" t="inlineStr">
         <is>
@@ -4167,15 +4167,15 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>fc_cooling_exhaust_plenum_gap_actual</t>
+          <t>fc_cooling_inlet_ramp_angle</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>3.300000000000004</v>
+        <v>2.694284289856101</v>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>deg</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -4187,15 +4187,15 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>fc_cooling_inlet_plenum_gap_min</t>
+          <t>fc_cooling_inlet_sidewall_angle</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>deg</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -4207,11 +4207,11 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>fc_cooling_exhaust_plenum_gap_min</t>
+          <t>fc_cooling_inlet_lip_radius</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C189" t="inlineStr">
         <is>
@@ -4227,11 +4227,11 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>fc_cooling_min_fuselage_width</t>
+          <t>fc_cooling_exhaust_center_x</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>142.4</v>
+        <v>255.25</v>
       </c>
       <c r="C190" t="inlineStr">
         <is>
@@ -4247,11 +4247,11 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>fc_cooling_section_joint_edge_distance</t>
+          <t>fc_cooling_exhaust_center_y</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>12</v>
+        <v>74.50000000000001</v>
       </c>
       <c r="C191" t="inlineStr">
         <is>
@@ -4267,11 +4267,11 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>fc_cooling_grille_corner_radius</t>
+          <t>fc_cooling_exhaust_center_z</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>4</v>
+        <v>-33.10930732488546</v>
       </c>
       <c r="C192" t="inlineStr">
         <is>
@@ -4287,11 +4287,11 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>fc_cooling_min_web_between_slots</t>
+          <t>fc_cooling_exhaust_panel_length</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>3</v>
+        <v>180</v>
       </c>
       <c r="C193" t="inlineStr">
         <is>
@@ -4307,17 +4307,15 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>fc_cooling_exhaust_grille_fastener</t>
-        </is>
-      </c>
-      <c r="B194" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
+          <t>fc_cooling_exhaust_panel_height</t>
+        </is>
+      </c>
+      <c r="B194" t="n">
+        <v>111</v>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -4329,31 +4327,31 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>general_print_tolerance</t>
+          <t>fc_cooling_exhaust_slot_count</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>0.3</v>
+        <v>12</v>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>unitless</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>User CAD tolerance/clearance</t>
+          <t>H2AIR CAD export</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>transition_fit_clearance</t>
+          <t>fc_cooling_exhaust_slot_length</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>0.24</v>
+        <v>180</v>
       </c>
       <c r="C196" t="inlineStr">
         <is>
@@ -4362,18 +4360,18 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>User CAD tolerance/clearance</t>
+          <t>H2AIR CAD export</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>carbon_tube_fit_clearance</t>
+          <t>fc_cooling_exhaust_slot_width</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>0.5</v>
+        <v>6.5</v>
       </c>
       <c r="C197" t="inlineStr">
         <is>
@@ -4382,14 +4380,14 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>User CAD tolerance/clearance</t>
+          <t>H2AIR CAD export</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>component_keepout_clearance</t>
+          <t>fc_cooling_exhaust_slot_gap</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -4402,18 +4400,18 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>User CAD tolerance/clearance</t>
+          <t>H2AIR CAD export</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>prop_disk_edge_clearance</t>
+          <t>fc_cooling_exhaust_shroud_depth</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C199" t="inlineStr">
         <is>
@@ -4422,80 +4420,78 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>User CAD tolerance/clearance</t>
+          <t>H2AIR CAD export</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>bolt_pocket_diameter_clearance</t>
+          <t>fc_cooling_exhaust_louvre_angle</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>1.7</v>
+        <v>15</v>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>deg</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>User CAD tolerance/clearance</t>
+          <t>H2AIR CAD export</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>default_motor_mount_fastener</t>
-        </is>
-      </c>
-      <c r="B201" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
+          <t>fc_cooling_exhaust_lip_radius</t>
+        </is>
+      </c>
+      <c r="B201" t="n">
+        <v>2</v>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>User CAD fastener parameter</t>
+          <t>H2AIR CAD export</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>bolt_M3_OD</t>
+          <t>fc_cooling_fan_count</t>
         </is>
       </c>
       <c r="B202" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>unitless</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>User CAD fastener parameter</t>
+          <t>H2AIR CAD export</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>bolt_M3_clearance_hole_OD</t>
+          <t>fc_cooling_fan_diameter</t>
         </is>
       </c>
       <c r="B203" t="n">
-        <v>3.2</v>
+        <v>80</v>
       </c>
       <c r="C203" t="inlineStr">
         <is>
@@ -4504,18 +4500,18 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>User CAD fastener parameter</t>
+          <t>H2AIR CAD export</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>bolt_M3_head_OD</t>
+          <t>fc_cooling_fan_center_spacing</t>
         </is>
       </c>
       <c r="B204" t="n">
-        <v>6.5</v>
+        <v>86</v>
       </c>
       <c r="C204" t="inlineStr">
         <is>
@@ -4524,18 +4520,18 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>User CAD fastener parameter</t>
+          <t>H2AIR CAD export</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>bolt_M4_OD</t>
+          <t>fc_cooling_fan_1_center_x</t>
         </is>
       </c>
       <c r="B205" t="n">
-        <v>4</v>
+        <v>212.2500000000001</v>
       </c>
       <c r="C205" t="inlineStr">
         <is>
@@ -4544,18 +4540,18 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>User CAD fastener parameter</t>
+          <t>H2AIR CAD export</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>bolt_M4_clearance_hole_OD</t>
+          <t>fc_cooling_fan_2_center_x</t>
         </is>
       </c>
       <c r="B206" t="n">
-        <v>4.2</v>
+        <v>298.25</v>
       </c>
       <c r="C206" t="inlineStr">
         <is>
@@ -4564,18 +4560,18 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>User CAD fastener parameter</t>
+          <t>H2AIR CAD export</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>bolt_M4_head_OD</t>
+          <t>fc_cooling_fan_center_y</t>
         </is>
       </c>
       <c r="B207" t="n">
-        <v>8.220000000000001</v>
+        <v>74.50000000000001</v>
       </c>
       <c r="C207" t="inlineStr">
         <is>
@@ -4584,18 +4580,18 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>User CAD fastener parameter</t>
+          <t>H2AIR CAD export</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>bolt_M5_OD</t>
+          <t>fc_cooling_fan_center_z</t>
         </is>
       </c>
       <c r="B208" t="n">
-        <v>5</v>
+        <v>-33.10930732488546</v>
       </c>
       <c r="C208" t="inlineStr">
         <is>
@@ -4604,18 +4600,18 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>User CAD fastener parameter</t>
+          <t>H2AIR CAD export</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>bolt_M5_clearance_hole_OD</t>
+          <t>fc_cooling_inlet_plenum_gap_actual</t>
         </is>
       </c>
       <c r="B209" t="n">
-        <v>5.2</v>
+        <v>10.30000000000002</v>
       </c>
       <c r="C209" t="inlineStr">
         <is>
@@ -4624,18 +4620,18 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>User CAD fastener parameter</t>
+          <t>H2AIR CAD export</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>bolt_M5_head_OD</t>
+          <t>fc_cooling_exhaust_plenum_gap_actual</t>
         </is>
       </c>
       <c r="B210" t="n">
-        <v>9.720000000000001</v>
+        <v>10.30000000000002</v>
       </c>
       <c r="C210" t="inlineStr">
         <is>
@@ -4644,22 +4640,22 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>User CAD fastener parameter</t>
+          <t>H2AIR CAD export</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>wing_rib_count</t>
+          <t>fc_cooling_inlet_plenum_gap_min</t>
         </is>
       </c>
       <c r="B211" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>unitless</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
@@ -4671,15 +4667,15 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>horizontal_tail_rib_count</t>
+          <t>fc_cooling_exhaust_plenum_gap_min</t>
         </is>
       </c>
       <c r="B212" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>unitless</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
@@ -4691,18 +4687,482 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
+          <t>fc_cooling_min_fuselage_width</t>
+        </is>
+      </c>
+      <c r="B213" t="n">
+        <v>142.4</v>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>H2AIR CAD export</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>fc_cooling_section_joint_edge_distance</t>
+        </is>
+      </c>
+      <c r="B214" t="n">
+        <v>12</v>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>H2AIR CAD export</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>fc_cooling_grille_corner_radius</t>
+        </is>
+      </c>
+      <c r="B215" t="n">
+        <v>4</v>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>H2AIR CAD export</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>fc_cooling_min_web_between_slots</t>
+        </is>
+      </c>
+      <c r="B216" t="n">
+        <v>3</v>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>H2AIR CAD export</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>fc_cooling_exhaust_grille_fastener</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>H2AIR CAD export</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>general_print_tolerance</t>
+        </is>
+      </c>
+      <c r="B218" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>User CAD tolerance/clearance</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>transition_fit_clearance</t>
+        </is>
+      </c>
+      <c r="B219" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>User CAD tolerance/clearance</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>carbon_tube_fit_clearance</t>
+        </is>
+      </c>
+      <c r="B220" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>User CAD tolerance/clearance</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>component_keepout_clearance</t>
+        </is>
+      </c>
+      <c r="B221" t="n">
+        <v>3</v>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>User CAD tolerance/clearance</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>prop_disk_edge_clearance</t>
+        </is>
+      </c>
+      <c r="B222" t="n">
+        <v>20</v>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>User CAD tolerance/clearance</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>bolt_pocket_diameter_clearance</t>
+        </is>
+      </c>
+      <c r="B223" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>User CAD tolerance/clearance</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>default_motor_mount_fastener</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>User CAD fastener parameter</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>bolt_M3_OD</t>
+        </is>
+      </c>
+      <c r="B225" t="n">
+        <v>3</v>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>User CAD fastener parameter</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>bolt_M3_clearance_hole_OD</t>
+        </is>
+      </c>
+      <c r="B226" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>User CAD fastener parameter</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>bolt_M3_head_OD</t>
+        </is>
+      </c>
+      <c r="B227" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>User CAD fastener parameter</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>bolt_M4_OD</t>
+        </is>
+      </c>
+      <c r="B228" t="n">
+        <v>4</v>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>User CAD fastener parameter</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>bolt_M4_clearance_hole_OD</t>
+        </is>
+      </c>
+      <c r="B229" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>User CAD fastener parameter</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>bolt_M4_head_OD</t>
+        </is>
+      </c>
+      <c r="B230" t="n">
+        <v>8.220000000000001</v>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>User CAD fastener parameter</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>bolt_M5_OD</t>
+        </is>
+      </c>
+      <c r="B231" t="n">
+        <v>5</v>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>User CAD fastener parameter</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>bolt_M5_clearance_hole_OD</t>
+        </is>
+      </c>
+      <c r="B232" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>User CAD fastener parameter</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>bolt_M5_head_OD</t>
+        </is>
+      </c>
+      <c r="B233" t="n">
+        <v>9.720000000000001</v>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>User CAD fastener parameter</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>wing_rib_count</t>
+        </is>
+      </c>
+      <c r="B234" t="n">
+        <v>16</v>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>unitless</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>H2AIR CAD export</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>horizontal_tail_rib_count</t>
+        </is>
+      </c>
+      <c r="B235" t="n">
+        <v>8</v>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>unitless</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>H2AIR CAD export</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
           <t>vertical_tail_rib_count_each</t>
         </is>
       </c>
-      <c r="B213" t="n">
-        <v>4</v>
-      </c>
-      <c r="C213" t="inlineStr">
+      <c r="B236" t="n">
+        <v>6</v>
+      </c>
+      <c r="C236" t="inlineStr">
         <is>
           <t>unitless</t>
         </is>
       </c>
-      <c r="D213" t="inlineStr">
+      <c r="D236" t="inlineStr">
         <is>
           <t>H2AIR CAD export</t>
         </is>

</xml_diff>

<commit_message>
Regenerate latest output with AutoSize Main Wing
Synchronize outputs/latest with the live-M2 coupled main-wing autosizing result.
</commit_message>
<xml_diff>
--- a/outputs/latest/details/params.xlsx
+++ b/outputs/latest/details/params.xlsx
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>3600</v>
+        <v>3359.385380530533</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -913,7 +913,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1800</v>
+        <v>1679.692690265266</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -933,7 +933,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>310</v>
+        <v>301.6702248753886</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -953,7 +953,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>190</v>
+        <v>224.2499624918836</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>254.8</v>
+        <v>264.8595888198138</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -993,7 +993,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>392.014</v>
+        <v>389.4991027950466</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1033,7 +1033,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>86.00930732488546</v>
+        <v>87.00930732488546</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1053,7 +1053,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>46.5</v>
+        <v>45.25053373130829</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1073,7 +1073,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>0.6129032258064516</v>
+        <v>0.743361273339173</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1195,7 +1195,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1215,7 +1215,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1295,7 +1295,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1415,7 +1415,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>4.750000000000004</v>
+        <v>4.37473313434586</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>915.9221570593505</v>
+        <v>934.505810950418</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -1455,7 +1455,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>457.9610785296753</v>
+        <v>467.252905475209</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -1575,7 +1575,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>86.00930732488546</v>
+        <v>87.00930732488546</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -1657,7 +1657,7 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -1677,7 +1677,7 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -1737,7 +1737,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>533.0190749553177</v>
+        <v>488.210642814369</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -2079,7 +2079,7 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>86.00930732488546</v>
+        <v>87.00930732488546</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -2159,7 +2159,7 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>-243.1156926751145</v>
+        <v>-241.4909595407687</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -2259,7 +2259,7 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>305.875</v>
+        <v>305.8749999999999</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
@@ -2339,7 +2339,7 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>-243.1156926751145</v>
+        <v>-241.4909595407687</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
@@ -2359,7 +2359,7 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>129.1063853502291</v>
+        <v>127.4816522158832</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
@@ -2379,7 +2379,7 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>455.7139999999999</v>
+        <v>455.714</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
@@ -2419,7 +2419,7 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>62.75930732488547</v>
+        <v>64.38404045923131</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
@@ -2439,7 +2439,7 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>-243.1156926751145</v>
+        <v>-241.4909595407687</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
@@ -2459,7 +2459,7 @@
         </is>
       </c>
       <c r="B102" t="n">
-        <v>305.875</v>
+        <v>305.8749999999999</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
@@ -2479,7 +2479,7 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>455.7139999999999</v>
+        <v>455.714</v>
       </c>
       <c r="C103" t="inlineStr">
         <is>
@@ -2519,7 +2519,7 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>62.75930732488547</v>
+        <v>64.38404045923131</v>
       </c>
       <c r="C105" t="inlineStr">
         <is>
@@ -2539,7 +2539,7 @@
         </is>
       </c>
       <c r="B106" t="n">
-        <v>-243.1156926751145</v>
+        <v>-241.4909595407687</v>
       </c>
       <c r="C106" t="inlineStr">
         <is>
@@ -2559,7 +2559,7 @@
         </is>
       </c>
       <c r="B107" t="n">
-        <v>305.875</v>
+        <v>305.8749999999999</v>
       </c>
       <c r="C107" t="inlineStr">
         <is>
@@ -2639,7 +2639,7 @@
         </is>
       </c>
       <c r="B111" t="n">
-        <v>56.28430732488547</v>
+        <v>57.90904045923131</v>
       </c>
       <c r="C111" t="inlineStr">
         <is>
@@ -5115,7 +5115,7 @@
         </is>
       </c>
       <c r="B234" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C234" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Regenerate latest output with inspection flight envelope
Synchronize outputs/latest with the tested inspection manoeuvre and gust-stall constrained design.
</commit_message>
<xml_diff>
--- a/outputs/latest/details/params.xlsx
+++ b/outputs/latest/details/params.xlsx
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>3359.385380530533</v>
+        <v>3383.421255562335</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -913,7 +913,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1679.692690265266</v>
+        <v>1691.710627781167</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -933,7 +933,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>301.6702248753886</v>
+        <v>331.0711281167754</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -953,7 +953,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>224.2499624918836</v>
+        <v>241.807183206562</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>264.8595888198138</v>
+        <v>288.7572895781391</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -993,7 +993,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>389.4991027950466</v>
+        <v>383.5246776054652</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1053,7 +1053,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>45.25053373130829</v>
+        <v>49.66066921751631</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1073,7 +1073,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>0.743361273339173</v>
+        <v>0.73037834673784</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1415,7 +1415,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>4.37473313434586</v>
+        <v>2.16966539124186</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>934.505810950418</v>
+        <v>1117.732932249976</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -1455,7 +1455,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>467.252905475209</v>
+        <v>558.8664661249882</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -1737,7 +1737,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>488.210642814369</v>
+        <v>539.4389142995057</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -2099,7 +2099,7 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -2119,7 +2119,7 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -2159,7 +2159,7 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>-241.4909595407687</v>
+        <v>-243.6960272838726</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -2339,7 +2339,7 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>-241.4909595407687</v>
+        <v>-243.6960272838726</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
@@ -2359,7 +2359,7 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>127.4816522158832</v>
+        <v>129.6867199589872</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
@@ -2419,7 +2419,7 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>64.38404045923131</v>
+        <v>62.17897271612731</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
@@ -2439,7 +2439,7 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>-241.4909595407687</v>
+        <v>-243.6960272838726</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
@@ -2519,7 +2519,7 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>64.38404045923131</v>
+        <v>62.17897271612731</v>
       </c>
       <c r="C105" t="inlineStr">
         <is>
@@ -2539,7 +2539,7 @@
         </is>
       </c>
       <c r="B106" t="n">
-        <v>-241.4909595407687</v>
+        <v>-243.6960272838726</v>
       </c>
       <c r="C106" t="inlineStr">
         <is>
@@ -2639,7 +2639,7 @@
         </is>
       </c>
       <c r="B111" t="n">
-        <v>57.90904045923131</v>
+        <v>55.70397271612731</v>
       </c>
       <c r="C111" t="inlineStr">
         <is>
@@ -5135,7 +5135,7 @@
         </is>
       </c>
       <c r="B235" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C235" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Regenerate latest output with tail planform autosizing
Synchronize outputs/latest with the tested coupled horizontal- and vertical-tail planform autosizing result.
</commit_message>
<xml_diff>
--- a/outputs/latest/details/params.xlsx
+++ b/outputs/latest/details/params.xlsx
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>1117.732932249976</v>
+        <v>965.4126607604868</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -1455,7 +1455,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>558.8664661249882</v>
+        <v>482.7063303802434</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -1475,7 +1475,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>218</v>
+        <v>268.1701835445797</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -1495,7 +1495,7 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>152.6</v>
+        <v>160.9021101267478</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -1515,7 +1515,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>187.2235294117647</v>
+        <v>219.00564989474</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -1535,7 +1535,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>1003.420117647059</v>
+        <v>995.4745875263151</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>26.16</v>
+        <v>32.18042202534956</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -1615,7 +1615,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -1737,7 +1737,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>539.4389142995057</v>
+        <v>399.5921904049848</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -1757,7 +1757,7 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>148</v>
+        <v>199.7960952024924</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -1777,7 +1777,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>88.79999999999998</v>
+        <v>119.8776571214954</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -1797,7 +1797,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>1080.074333333333</v>
+        <v>1069.499297229491</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -1837,7 +1837,7 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>17.76</v>
+        <v>23.97553142429909</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -5135,7 +5135,7 @@
         </is>
       </c>
       <c r="B235" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C235" t="inlineStr">
         <is>
@@ -5155,7 +5155,7 @@
         </is>
       </c>
       <c r="B236" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C236" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Synchronize performance-constrained tail outputs
Update outputs/latest to the merged performance-constrained tail sizing result.
</commit_message>
<xml_diff>
--- a/outputs/latest/details/params.xlsx
+++ b/outputs/latest/details/params.xlsx
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>965.4126607604868</v>
+        <v>917.891874978866</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -1455,7 +1455,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>482.7063303802434</v>
+        <v>458.945937489433</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -1475,7 +1475,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>268.1701835445797</v>
+        <v>253.2610232535541</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -1495,7 +1495,7 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>160.9021101267478</v>
+        <v>149.5279569590623</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -1515,7 +1515,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>219.00564989474</v>
+        <v>205.8470072519599</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -1535,7 +1535,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>995.4745875263151</v>
+        <v>998.7642481870101</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>32.18042202534956</v>
+        <v>30.39132279042649</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -1615,7 +1615,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>0.6</v>
+        <v>0.5904104588938714</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -1737,7 +1737,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>399.5921904049848</v>
+        <v>394.2680025405157</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -1757,7 +1757,7 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>199.7960952024924</v>
+        <v>177.0671917201751</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -1777,7 +1777,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>119.8776571214954</v>
+        <v>97.05451850599299</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -1797,7 +1797,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>1069.499297229491</v>
+        <v>1075.052674091233</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -1837,7 +1837,7 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>23.97553142429909</v>
+        <v>21.24806300642101</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -1857,7 +1857,7 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>0.6</v>
+        <v>0.5481225379084983</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Sync generated AVL outputs
</commit_message>
<xml_diff>
--- a/outputs/latest/details/params.xlsx
+++ b/outputs/latest/details/params.xlsx
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>3383.421255562335</v>
+        <v>3338.674826810574</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -913,7 +913,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1691.710627781167</v>
+        <v>1669.337413405287</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -933,7 +933,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>331.0711281167754</v>
+        <v>365.2136021641022</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -953,7 +953,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>241.807183206562</v>
+        <v>241.3318068585455</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>288.7572895781391</v>
+        <v>307.4896735350876</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -993,7 +993,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>383.5246776054652</v>
+        <v>378.8415816162281</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1033,7 +1033,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>87.00930732488546</v>
+        <v>86.6182871625778</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1053,7 +1053,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>49.66066921751631</v>
+        <v>54.78204032461533</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1073,7 +1073,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>0.73037834673784</v>
+        <v>0.6607963269399461</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1415,7 +1415,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>2.16966539124186</v>
+        <v>0</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>917.891874978866</v>
+        <v>829.6142227057785</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -1455,7 +1455,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>458.945937489433</v>
+        <v>414.8071113528893</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -1475,7 +1475,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>253.2610232535541</v>
+        <v>180.527816071069</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -1495,7 +1495,7 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>149.5279569590623</v>
+        <v>136.3310121288753</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -1515,7 +1515,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>205.8470072519599</v>
+        <v>159.4568734945347</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -1535,7 +1535,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>998.7642481870101</v>
+        <v>1010.361781626366</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -1575,7 +1575,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>87.00930732488546</v>
+        <v>86.6182871625778</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>30.39132279042649</v>
+        <v>21.66333792852828</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -1615,7 +1615,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>0.5904104588938714</v>
+        <v>0.7551800885643319</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -1657,7 +1657,7 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -1677,7 +1677,7 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -1737,7 +1737,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>394.2680025405157</v>
+        <v>324.8112125229393</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -1757,7 +1757,7 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>177.0671917201751</v>
+        <v>161.203277498156</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -1777,7 +1777,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>97.05451850599299</v>
+        <v>87.89222743549932</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -1797,7 +1797,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>1075.052674091233</v>
+        <v>1078.255057626753</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -1837,7 +1837,7 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>21.24806300642101</v>
+        <v>19.34439329977872</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -1857,7 +1857,7 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>0.5481225379084983</v>
+        <v>0.5452260574323913</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
@@ -1899,7 +1899,7 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
@@ -1919,7 +1919,7 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
@@ -2079,7 +2079,7 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>87.00930732488546</v>
+        <v>86.6182871625778</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -2099,7 +2099,7 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -2119,7 +2119,7 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -2159,7 +2159,7 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>-243.6960272838726</v>
+        <v>-246.6477329997298</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -2339,7 +2339,7 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>-243.6960272838726</v>
+        <v>-246.6477329997298</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
@@ -2359,7 +2359,7 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>129.6867199589872</v>
+        <v>132.6384256748443</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
@@ -2419,7 +2419,7 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>62.17897271612731</v>
+        <v>59.22726700027013</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
@@ -2439,7 +2439,7 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>-243.6960272838726</v>
+        <v>-246.6477329997298</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
@@ -2519,7 +2519,7 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>62.17897271612731</v>
+        <v>59.22726700027013</v>
       </c>
       <c r="C105" t="inlineStr">
         <is>
@@ -2539,7 +2539,7 @@
         </is>
       </c>
       <c r="B106" t="n">
-        <v>-243.6960272838726</v>
+        <v>-246.6477329997298</v>
       </c>
       <c r="C106" t="inlineStr">
         <is>
@@ -2639,7 +2639,7 @@
         </is>
       </c>
       <c r="B111" t="n">
-        <v>55.70397271612731</v>
+        <v>52.75226700027013</v>
       </c>
       <c r="C111" t="inlineStr">
         <is>
@@ -5135,7 +5135,7 @@
         </is>
       </c>
       <c r="B235" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C235" t="inlineStr">
         <is>
@@ -5155,7 +5155,7 @@
         </is>
       </c>
       <c r="B236" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C236" t="inlineStr">
         <is>

</xml_diff>